<commit_message>
change big in project with medo
</commit_message>
<xml_diff>
--- a/documents/tests/checkList_anbara_test.xlsx
+++ b/documents/tests/checkList_anbara_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon6\www\anbara\documents\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729B6ACB-CAAA-458E-9E7B-6553DCE21393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C2D909-E3FF-416A-889F-7529BF1DBFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7EFB61C1-2B40-49A4-B058-302E36BE4D17}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="249">
   <si>
     <t>چک لیست</t>
   </si>
@@ -1935,46 +1935,58 @@
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
     </row>
-    <row r="85" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="85" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A85" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B85" s="3"/>
+      <c r="B85" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C85" s="3"/>
     </row>
-    <row r="86" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="86" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A86" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B86" s="3"/>
+      <c r="B86" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C86" s="3"/>
     </row>
-    <row r="87" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="87" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A87" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B87" s="3"/>
+      <c r="B87" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C87" s="3"/>
     </row>
-    <row r="88" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="88" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A88" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B88" s="3"/>
+      <c r="B88" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C88" s="3"/>
     </row>
-    <row r="89" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="89" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A89" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B89" s="3"/>
+      <c r="B89" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C89" s="3"/>
     </row>
-    <row r="90" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="90" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A90" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B90" s="3"/>
+      <c r="B90" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C90" s="3"/>
     </row>
     <row r="91" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
@@ -1984,53 +1996,67 @@
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
     </row>
-    <row r="92" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="92" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A92" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B92" s="3"/>
+      <c r="B92" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C92" s="3"/>
     </row>
-    <row r="93" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="93" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A93" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B93" s="3"/>
+      <c r="B93" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C93" s="3"/>
     </row>
-    <row r="94" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="94" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A94" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B94" s="3"/>
+      <c r="B94" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C94" s="3"/>
     </row>
-    <row r="95" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="95" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A95" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B95" s="3"/>
+      <c r="B95" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C95" s="3"/>
     </row>
-    <row r="96" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="96" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A96" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B96" s="3"/>
+      <c r="B96" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C96" s="3"/>
     </row>
-    <row r="97" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="97" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A97" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B97" s="3"/>
+      <c r="B97" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C97" s="3"/>
     </row>
-    <row r="98" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="98" spans="1:3" s="1" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A98" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B98" s="3"/>
+      <c r="B98" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C98" s="3"/>
     </row>
     <row r="99" spans="1:3" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.5">

</xml_diff>